<commit_message>
ça a buggé ?
</commit_message>
<xml_diff>
--- a/Pharmacologie special/data/Maladies.xlsx
+++ b/Pharmacologie special/data/Maladies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moito\Desktop\Sérieux\Projet\Site web\Pharmacologie special\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1529574E-F5F3-4432-9696-EF9A300A1D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6C6EF5B-1545-4907-8D8D-8099CFAC3D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{550D4594-D7DD-4F67-887A-DCF2F0E62F5B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="209">
   <si>
     <t>Pathologie</t>
   </si>
@@ -663,6 +663,9 @@
   </si>
   <si>
     <t>2eme intention_2</t>
+  </si>
+  <si>
+    <t>a</t>
   </si>
 </sst>
 </file>
@@ -2041,6 +2044,9 @@
       <c r="D51" t="s">
         <v>189</v>
       </c>
+      <c r="E51" t="s">
+        <v>208</v>
+      </c>
       <c r="K51" t="s">
         <v>190</v>
       </c>

</xml_diff>